<commit_message>
Atualizando o arquivo XLSX
</commit_message>
<xml_diff>
--- a/Jogos_do_Dia_Betfair_Back_Lay_2026-09-15.xlsx
+++ b/Jogos_do_Dia_Betfair_Back_Lay_2026-09-15.xlsx
@@ -475,7 +475,7 @@
     <t>Real Madrid</t>
   </si>
   <si>
-    <t>2026-09-13 07:13:58</t>
+    <t>2026-09-13 09:38:58</t>
   </si>
 </sst>
 </file>
@@ -1072,10 +1072,10 @@
         <v>1.44</v>
       </c>
       <c r="G2">
-        <v>1.54</v>
+        <v>1.53</v>
       </c>
       <c r="H2">
-        <v>9.6</v>
+        <v>9.4</v>
       </c>
       <c r="I2">
         <v>18</v>
@@ -1084,7 +1084,7 @@
         <v>3.85</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="L2">
         <v>1.49</v>
@@ -1096,7 +1096,7 @@
         <v>2.7</v>
       </c>
       <c r="O2">
-        <v>1.44</v>
+        <v>1.45</v>
       </c>
       <c r="P2">
         <v>1.58</v>
@@ -1105,10 +1105,10 @@
         <v>2.28</v>
       </c>
       <c r="R2">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="S2">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="T2">
         <v>2.52</v>
@@ -1120,10 +1120,10 @@
         <v>1.09</v>
       </c>
       <c r="W2">
-        <v>2.84</v>
+        <v>2.9</v>
       </c>
       <c r="X2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="Y2">
         <v>1000</v>
@@ -1135,10 +1135,10 @@
         <v>1000</v>
       </c>
       <c r="AB2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="AC2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="AD2">
         <v>1000</v>
@@ -1147,10 +1147,10 @@
         <v>1000</v>
       </c>
       <c r="AF2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="AG2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="AH2">
         <v>1000</v>
@@ -1159,7 +1159,7 @@
         <v>1000</v>
       </c>
       <c r="AJ2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="AK2">
         <v>1000</v>
@@ -1171,7 +1171,7 @@
         <v>1000</v>
       </c>
       <c r="AN2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="AO2">
         <v>1000</v>
@@ -1231,7 +1231,7 @@
         <v>1.94</v>
       </c>
       <c r="BH2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="BI2">
         <v>2.54</v>
@@ -1249,7 +1249,7 @@
         <v>1.01</v>
       </c>
       <c r="BN2">
-        <v>690</v>
+        <v>570</v>
       </c>
       <c r="BO2">
         <v>2.96</v>
@@ -1317,7 +1317,7 @@
         <v>2.84</v>
       </c>
       <c r="H3">
-        <v>2.86</v>
+        <v>2.84</v>
       </c>
       <c r="I3">
         <v>3.55</v>
@@ -1326,7 +1326,7 @@
         <v>2.94</v>
       </c>
       <c r="K3">
-        <v>3.85</v>
+        <v>3.7</v>
       </c>
       <c r="L3">
         <v>1.52</v>
@@ -1335,13 +1335,13 @@
         <v>1.1</v>
       </c>
       <c r="N3">
-        <v>2.72</v>
+        <v>2.96</v>
       </c>
       <c r="O3">
         <v>1.47</v>
       </c>
       <c r="P3">
-        <v>1.58</v>
+        <v>1.57</v>
       </c>
       <c r="Q3">
         <v>2.32</v>
@@ -1553,61 +1553,61 @@
         <v>131</v>
       </c>
       <c r="F4">
-        <v>1.39</v>
+        <v>1.41</v>
       </c>
       <c r="G4">
-        <v>1.51</v>
+        <v>1.46</v>
       </c>
       <c r="H4">
-        <v>7.2</v>
+        <v>10</v>
       </c>
       <c r="I4">
-        <v>22</v>
+        <v>13.5</v>
       </c>
       <c r="J4">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="K4">
-        <v>5.8</v>
+        <v>5.1</v>
       </c>
       <c r="L4">
         <v>1.01</v>
       </c>
       <c r="M4">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="N4">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="O4">
         <v>1.34</v>
       </c>
       <c r="P4">
-        <v>1.81</v>
+        <v>1.9</v>
       </c>
       <c r="Q4">
-        <v>1.96</v>
+        <v>2.02</v>
       </c>
       <c r="R4">
-        <v>1.31</v>
+        <v>1.32</v>
       </c>
       <c r="S4">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="T4">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="U4">
-        <v>1.6</v>
+        <v>1.66</v>
       </c>
       <c r="V4">
-        <v>1.06</v>
+        <v>1.09</v>
       </c>
       <c r="W4">
-        <v>2.96</v>
+        <v>3.15</v>
       </c>
       <c r="X4">
-        <v>1000</v>
+        <v>970</v>
       </c>
       <c r="Y4">
         <v>36</v>
@@ -1664,55 +1664,55 @@
         <v>1.87</v>
       </c>
       <c r="AQ4">
-        <v>1.77</v>
+        <v>1.98</v>
       </c>
       <c r="AR4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="AS4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="AT4">
         <v>5.7</v>
       </c>
       <c r="AU4">
-        <v>7.4</v>
+        <v>2.08</v>
       </c>
       <c r="AV4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="AW4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="AX4">
-        <v>1.51</v>
+        <v>1.66</v>
       </c>
       <c r="AY4">
         <v>7.4</v>
       </c>
       <c r="AZ4">
-        <v>1.79</v>
+        <v>1.99</v>
       </c>
       <c r="BA4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="BB4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="BC4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="BD4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="BE4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="BF4">
-        <v>1.55</v>
+        <v>1.7</v>
       </c>
       <c r="BG4">
-        <v>1.87</v>
+        <v>2.08</v>
       </c>
       <c r="BH4">
         <v>1000</v>
@@ -1798,10 +1798,10 @@
         <v>1.87</v>
       </c>
       <c r="G5">
-        <v>2.1</v>
+        <v>2.08</v>
       </c>
       <c r="H5">
-        <v>3.7</v>
+        <v>3.85</v>
       </c>
       <c r="I5">
         <v>4.7</v>
@@ -1828,13 +1828,13 @@
         <v>2.04</v>
       </c>
       <c r="Q5">
-        <v>1.75</v>
+        <v>1.78</v>
       </c>
       <c r="R5">
         <v>1.39</v>
       </c>
       <c r="S5">
-        <v>2.88</v>
+        <v>2.92</v>
       </c>
       <c r="T5">
         <v>1.66</v>
@@ -1846,7 +1846,7 @@
         <v>1.27</v>
       </c>
       <c r="W5">
-        <v>1.91</v>
+        <v>1.92</v>
       </c>
       <c r="X5">
         <v>1000</v>
@@ -2040,7 +2040,7 @@
         <v>4.2</v>
       </c>
       <c r="G6">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H6">
         <v>2.12</v>
@@ -2049,7 +2049,7 @@
         <v>2.44</v>
       </c>
       <c r="J6">
-        <v>2.76</v>
+        <v>2.8</v>
       </c>
       <c r="K6">
         <v>3.45</v>
@@ -2067,10 +2067,10 @@
         <v>0</v>
       </c>
       <c r="P6">
-        <v>1.35</v>
+        <v>1.37</v>
       </c>
       <c r="Q6">
-        <v>2.92</v>
+        <v>2.96</v>
       </c>
       <c r="R6">
         <v>0</v>
@@ -2279,16 +2279,16 @@
         <v>134</v>
       </c>
       <c r="F7">
-        <v>2.12</v>
+        <v>2.1</v>
       </c>
       <c r="G7">
-        <v>2.62</v>
+        <v>2.56</v>
       </c>
       <c r="H7">
         <v>3.6</v>
       </c>
       <c r="I7">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="J7">
         <v>2.96</v>
@@ -2312,7 +2312,7 @@
         <v>1.4</v>
       </c>
       <c r="Q7">
-        <v>2.42</v>
+        <v>2.46</v>
       </c>
       <c r="R7">
         <v>0</v>
@@ -2763,22 +2763,22 @@
         <v>136</v>
       </c>
       <c r="F9">
-        <v>1.75</v>
+        <v>1.82</v>
       </c>
       <c r="G9">
-        <v>1.99</v>
+        <v>1.98</v>
       </c>
       <c r="H9">
-        <v>1.1</v>
+        <v>3.7</v>
       </c>
       <c r="I9">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="J9">
         <v>3.5</v>
       </c>
       <c r="K9">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -2796,7 +2796,7 @@
         <v>2</v>
       </c>
       <c r="Q9">
-        <v>1.81</v>
+        <v>1.8</v>
       </c>
       <c r="R9">
         <v>0</v>
@@ -3005,22 +3005,22 @@
         <v>137</v>
       </c>
       <c r="F10">
-        <v>3.45</v>
+        <v>3.95</v>
       </c>
       <c r="G10">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="H10">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="I10">
-        <v>2.02</v>
+        <v>2.12</v>
       </c>
       <c r="J10">
-        <v>3.95</v>
+        <v>3.6</v>
       </c>
       <c r="K10">
-        <v>4.6</v>
+        <v>5.1</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -3035,10 +3035,10 @@
         <v>0</v>
       </c>
       <c r="P10">
-        <v>2.42</v>
+        <v>2.58</v>
       </c>
       <c r="Q10">
-        <v>1.49</v>
+        <v>1.01</v>
       </c>
       <c r="R10">
         <v>0</v>
@@ -3247,7 +3247,7 @@
         <v>138</v>
       </c>
       <c r="F11">
-        <v>1.89</v>
+        <v>1.88</v>
       </c>
       <c r="G11">
         <v>2</v>
@@ -3259,10 +3259,10 @@
         <v>4.1</v>
       </c>
       <c r="J11">
-        <v>3.9</v>
+        <v>3.95</v>
       </c>
       <c r="K11">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -3280,7 +3280,7 @@
         <v>2.58</v>
       </c>
       <c r="Q11">
-        <v>1.46</v>
+        <v>1.5</v>
       </c>
       <c r="R11">
         <v>0</v>
@@ -3489,22 +3489,22 @@
         <v>139</v>
       </c>
       <c r="F12">
-        <v>1.45</v>
+        <v>1.41</v>
       </c>
       <c r="G12">
-        <v>1.68</v>
+        <v>1.67</v>
       </c>
       <c r="H12">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="I12">
         <v>11</v>
       </c>
       <c r="J12">
-        <v>4.2</v>
+        <v>3.2</v>
       </c>
       <c r="K12">
-        <v>7.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -3519,10 +3519,10 @@
         <v>0</v>
       </c>
       <c r="P12">
-        <v>2.06</v>
+        <v>2.08</v>
       </c>
       <c r="Q12">
-        <v>1.6</v>
+        <v>1.61</v>
       </c>
       <c r="R12">
         <v>0</v>
@@ -3731,22 +3731,22 @@
         <v>140</v>
       </c>
       <c r="F13">
-        <v>2.42</v>
+        <v>2.56</v>
       </c>
       <c r="G13">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="H13">
-        <v>2.42</v>
+        <v>2.46</v>
       </c>
       <c r="I13">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="J13">
-        <v>3.25</v>
+        <v>3.35</v>
       </c>
       <c r="K13">
-        <v>5.8</v>
+        <v>5</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -3761,10 +3761,10 @@
         <v>0</v>
       </c>
       <c r="P13">
-        <v>2.1</v>
+        <v>2.28</v>
       </c>
       <c r="Q13">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
       <c r="R13">
         <v>0</v>
@@ -3973,16 +3973,16 @@
         <v>141</v>
       </c>
       <c r="F14">
-        <v>2.14</v>
+        <v>2.18</v>
       </c>
       <c r="G14">
-        <v>2.18</v>
+        <v>2.22</v>
       </c>
       <c r="H14">
-        <v>3.85</v>
+        <v>3.8</v>
       </c>
       <c r="I14">
-        <v>3.95</v>
+        <v>3.9</v>
       </c>
       <c r="J14">
         <v>3.5</v>
@@ -4003,7 +4003,7 @@
         <v>1.35</v>
       </c>
       <c r="P14">
-        <v>1.86</v>
+        <v>1.89</v>
       </c>
       <c r="Q14">
         <v>2.06</v>
@@ -4036,10 +4036,10 @@
         <v>29</v>
       </c>
       <c r="AA14">
-        <v>1000</v>
+        <v>85</v>
       </c>
       <c r="AB14">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="AC14">
         <v>8</v>
@@ -4048,7 +4048,7 @@
         <v>16</v>
       </c>
       <c r="AE14">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="AF14">
         <v>13</v>
@@ -4060,10 +4060,10 @@
         <v>19</v>
       </c>
       <c r="AI14">
-        <v>920</v>
+        <v>610</v>
       </c>
       <c r="AJ14">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AK14">
         <v>25</v>
@@ -4102,7 +4102,7 @@
         <v>14</v>
       </c>
       <c r="AW14">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AX14">
         <v>11.5</v>
@@ -4117,7 +4117,7 @@
         <v>46</v>
       </c>
       <c r="BB14">
-        <v>17</v>
+        <v>17.5</v>
       </c>
       <c r="BC14">
         <v>20</v>
@@ -4215,22 +4215,22 @@
         <v>142</v>
       </c>
       <c r="F15">
-        <v>1.04</v>
+        <v>2.92</v>
       </c>
       <c r="G15">
-        <v>1000</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>1.04</v>
+        <v>2.22</v>
       </c>
       <c r="I15">
-        <v>1000</v>
+        <v>2.82</v>
       </c>
       <c r="J15">
-        <v>1.01</v>
+        <v>3.25</v>
       </c>
       <c r="K15">
-        <v>920</v>
+        <v>4.9</v>
       </c>
       <c r="L15">
         <v>0</v>
@@ -4245,10 +4245,10 @@
         <v>0</v>
       </c>
       <c r="P15">
-        <v>1.24</v>
+        <v>2.1</v>
       </c>
       <c r="Q15">
-        <v>1.01</v>
+        <v>1.49</v>
       </c>
       <c r="R15">
         <v>0</v>
@@ -4457,22 +4457,22 @@
         <v>143</v>
       </c>
       <c r="F16">
-        <v>1.04</v>
+        <v>2.54</v>
       </c>
       <c r="G16">
-        <v>1000</v>
+        <v>3.1</v>
       </c>
       <c r="H16">
-        <v>1.04</v>
+        <v>2.28</v>
       </c>
       <c r="I16">
-        <v>1000</v>
+        <v>2.7</v>
       </c>
       <c r="J16">
-        <v>1.01</v>
+        <v>3.25</v>
       </c>
       <c r="K16">
-        <v>920</v>
+        <v>6</v>
       </c>
       <c r="L16">
         <v>0</v>
@@ -4487,10 +4487,10 @@
         <v>0</v>
       </c>
       <c r="P16">
-        <v>1.24</v>
+        <v>2.52</v>
       </c>
       <c r="Q16">
-        <v>1.01</v>
+        <v>1.5</v>
       </c>
       <c r="R16">
         <v>0</v>
@@ -4729,7 +4729,7 @@
         <v>0</v>
       </c>
       <c r="P17">
-        <v>2.18</v>
+        <v>2.2</v>
       </c>
       <c r="Q17">
         <v>1.63</v>
@@ -4941,10 +4941,10 @@
         <v>145</v>
       </c>
       <c r="F18">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
       <c r="G18">
-        <v>2.12</v>
+        <v>2.18</v>
       </c>
       <c r="H18">
         <v>4.8</v>
@@ -4971,7 +4971,7 @@
         <v>0</v>
       </c>
       <c r="P18">
-        <v>1.47</v>
+        <v>1.5</v>
       </c>
       <c r="Q18">
         <v>2.64</v>
@@ -5186,19 +5186,19 @@
         <v>1.67</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>1.87</v>
       </c>
       <c r="H19">
-        <v>3.9</v>
+        <v>4.4</v>
       </c>
       <c r="I19">
-        <v>7.8</v>
+        <v>6.8</v>
       </c>
       <c r="J19">
-        <v>3.7</v>
+        <v>3.95</v>
       </c>
       <c r="K19">
-        <v>7</v>
+        <v>5.8</v>
       </c>
       <c r="L19">
         <v>0</v>
@@ -5213,10 +5213,10 @@
         <v>0</v>
       </c>
       <c r="P19">
-        <v>2</v>
+        <v>2.06</v>
       </c>
       <c r="Q19">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="R19">
         <v>0</v>
@@ -5434,7 +5434,7 @@
         <v>13.5</v>
       </c>
       <c r="I20">
-        <v>19.5</v>
+        <v>17.5</v>
       </c>
       <c r="J20">
         <v>8.6</v>
@@ -5667,37 +5667,37 @@
         <v>148</v>
       </c>
       <c r="F21">
-        <v>1.97</v>
+        <v>1.95</v>
       </c>
       <c r="G21">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="H21">
+        <v>5</v>
+      </c>
+      <c r="I21">
         <v>5.1</v>
       </c>
-      <c r="I21">
-        <v>5.3</v>
-      </c>
       <c r="J21">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="K21">
-        <v>3.4</v>
+        <v>3.45</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="M21">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="N21">
-        <v>3</v>
+        <v>3.05</v>
       </c>
       <c r="O21">
-        <v>1.47</v>
+        <v>1.46</v>
       </c>
       <c r="P21">
-        <v>1.67</v>
+        <v>1.68</v>
       </c>
       <c r="Q21">
         <v>2.38</v>
@@ -5706,13 +5706,13 @@
         <v>1.25</v>
       </c>
       <c r="S21">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="T21">
         <v>2.08</v>
       </c>
       <c r="U21">
-        <v>1.85</v>
+        <v>1.86</v>
       </c>
       <c r="V21">
         <v>0</v>
@@ -5745,7 +5745,7 @@
         <v>1000</v>
       </c>
       <c r="AF21">
-        <v>11.5</v>
+        <v>10.5</v>
       </c>
       <c r="AG21">
         <v>11</v>
@@ -5763,13 +5763,13 @@
         <v>25</v>
       </c>
       <c r="AL21">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="AM21">
         <v>1000</v>
       </c>
       <c r="AN21">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AO21">
         <v>1000</v>
@@ -5790,22 +5790,22 @@
         <v>6.6</v>
       </c>
       <c r="AU21">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="AV21">
-        <v>17.5</v>
+        <v>18</v>
       </c>
       <c r="AW21">
         <v>34</v>
       </c>
       <c r="AX21">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="AY21">
         <v>9.800000000000001</v>
       </c>
       <c r="AZ21">
-        <v>16.5</v>
+        <v>18.5</v>
       </c>
       <c r="BA21">
         <v>38</v>
@@ -5909,19 +5909,19 @@
         <v>149</v>
       </c>
       <c r="F22">
-        <v>1.1</v>
+        <v>1.04</v>
       </c>
       <c r="G22">
-        <v>3.25</v>
+        <v>3.05</v>
       </c>
       <c r="H22">
-        <v>2.36</v>
+        <v>2.58</v>
       </c>
       <c r="I22">
-        <v>3.15</v>
+        <v>3</v>
       </c>
       <c r="J22">
-        <v>3.25</v>
+        <v>3.2</v>
       </c>
       <c r="K22">
         <v>4.1</v>
@@ -5942,7 +5942,7 @@
         <v>2.04</v>
       </c>
       <c r="Q22">
-        <v>1.66</v>
+        <v>1.65</v>
       </c>
       <c r="R22">
         <v>0</v>
@@ -6151,13 +6151,13 @@
         <v>150</v>
       </c>
       <c r="F23">
+        <v>1.61</v>
+      </c>
+      <c r="G23">
         <v>1.62</v>
       </c>
-      <c r="G23">
-        <v>1.65</v>
-      </c>
       <c r="H23">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="I23">
         <v>6.2</v>
@@ -6393,13 +6393,13 @@
         <v>151</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>2.02</v>
       </c>
       <c r="G24">
-        <v>2.12</v>
+        <v>2.06</v>
       </c>
       <c r="H24">
-        <v>3.9</v>
+        <v>3.95</v>
       </c>
       <c r="I24">
         <v>4.2</v>
@@ -6408,7 +6408,7 @@
         <v>3.65</v>
       </c>
       <c r="K24">
-        <v>3.85</v>
+        <v>3.8</v>
       </c>
       <c r="L24">
         <v>0</v>
@@ -6635,22 +6635,22 @@
         <v>152</v>
       </c>
       <c r="F25">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="G25">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="H25">
-        <v>1.32</v>
+        <v>1.29</v>
       </c>
       <c r="I25">
-        <v>1.34</v>
+        <v>1.31</v>
       </c>
       <c r="J25">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
       <c r="K25">
-        <v>6.4</v>
+        <v>7</v>
       </c>
       <c r="L25">
         <v>0</v>
@@ -6659,28 +6659,28 @@
         <v>1.02</v>
       </c>
       <c r="N25">
-        <v>7.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="O25">
-        <v>1.13</v>
+        <v>1.12</v>
       </c>
       <c r="P25">
-        <v>3.2</v>
+        <v>3.25</v>
       </c>
       <c r="Q25">
-        <v>1.41</v>
+        <v>1.39</v>
       </c>
       <c r="R25">
-        <v>1.93</v>
+        <v>1.96</v>
       </c>
       <c r="S25">
-        <v>1.97</v>
+        <v>1.95</v>
       </c>
       <c r="T25">
-        <v>1.67</v>
+        <v>1.69</v>
       </c>
       <c r="U25">
-        <v>2.38</v>
+        <v>2.36</v>
       </c>
       <c r="V25">
         <v>0</v>
@@ -6689,25 +6689,25 @@
         <v>0</v>
       </c>
       <c r="X25">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="Y25">
-        <v>14</v>
+        <v>14.5</v>
       </c>
       <c r="Z25">
         <v>10.5</v>
       </c>
       <c r="AA25">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AB25">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="AC25">
-        <v>16</v>
+        <v>16.5</v>
       </c>
       <c r="AD25">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="AE25">
         <v>12</v>
@@ -6716,13 +6716,13 @@
         <v>1000</v>
       </c>
       <c r="AG25">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="AH25">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="AI25">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AJ25">
         <v>470</v>
@@ -6734,28 +6734,28 @@
         <v>110</v>
       </c>
       <c r="AM25">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="AN25">
         <v>1000</v>
       </c>
       <c r="AO25">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
       <c r="AP25">
         <v>32</v>
       </c>
       <c r="AQ25">
-        <v>12.5</v>
+        <v>13</v>
       </c>
       <c r="AR25">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="AS25">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="AT25">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AU25">
         <v>13.5</v>
@@ -6773,7 +6773,7 @@
         <v>29</v>
       </c>
       <c r="AZ25">
-        <v>19.5</v>
+        <v>21</v>
       </c>
       <c r="BA25">
         <v>21</v>
@@ -6785,7 +6785,7 @@
         <v>42</v>
       </c>
       <c r="BD25">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="BE25">
         <v>55</v>
@@ -6794,7 +6794,7 @@
         <v>40</v>
       </c>
       <c r="BG25">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="BH25">
         <v>970</v>
@@ -6839,7 +6839,7 @@
         <v>1.01</v>
       </c>
       <c r="BV25">
-        <v>1000</v>
+        <v>970</v>
       </c>
       <c r="BW25">
         <v>1.01</v>

</xml_diff>